<commit_message>
Renumeração dos capítulos do livro: os Caps. 0–27 passam a 1–28 em todo o material, e a planilha CAMPO_v0.0.xlsx foi gerada de novo (semente fixa; dados idênticos)
</commit_message>
<xml_diff>
--- a/material/CAMPO_v0.0.xlsx
+++ b/material/CAMPO_v0.0.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="LEIA-ME" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Ocorrencias" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Painel" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Unidades" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Equipe" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Listas" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Arquivo_2025" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LEIA-ME" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ocorrencias" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Painel" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unidades" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipe" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listas" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Arquivo_2025" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="Abertas">Painel!$B$3</definedName>
@@ -543,7 +543,7 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Arquivo de exemplo do livro Power Fx na Prática (Capítulo 0). Dados fictícios: pessoas e unidades inventadas.</t>
+          <t>Arquivo de exemplo do livro Power Fx na Prática (Capítulo 1). Dados fictícios: pessoas e unidades inventadas.</t>
         </is>
       </c>
     </row>

</xml_diff>